<commit_message>
Deleting Mess up plates
</commit_message>
<xml_diff>
--- a/Plates/nitrate_key.xlsx
+++ b/Plates/nitrate_key.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jaedonswanson/Desktop/School/MS/Research/Microplate/Plates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0487EB1C-5029-9441-9D0A-8398755B4365}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74D34686-64EB-4148-86A4-85FB9D313436}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" firstSheet="2" activeTab="10" xr2:uid="{B6428683-2A57-0F44-B42C-96122C72F6E2}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" firstSheet="2" activeTab="8" xr2:uid="{B6428683-2A57-0F44-B42C-96122C72F6E2}"/>
   </bookViews>
   <sheets>
     <sheet name="Format" sheetId="1" r:id="rId1"/>
@@ -22,8 +22,6 @@
     <sheet name="06192026_4" sheetId="9" r:id="rId7"/>
     <sheet name="06222026_1" sheetId="11" r:id="rId8"/>
     <sheet name="06222026_2" sheetId="12" r:id="rId9"/>
-    <sheet name="06242026_1" sheetId="13" r:id="rId10"/>
-    <sheet name="06242026_2" sheetId="14" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -49,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="72">
   <si>
     <t>A</t>
   </si>
@@ -265,18 +263,6 @@
   </si>
   <si>
     <t>elm-bridge_06012026</t>
-  </si>
-  <si>
-    <t>gcp-x5dilute_06212026</t>
-  </si>
-  <si>
-    <t>heron-resi-x5dilute_06212026</t>
-  </si>
-  <si>
-    <t>elm-school-x5dilute_06212026</t>
-  </si>
-  <si>
-    <t>heron-map-x5dilute_06212026</t>
   </si>
 </sst>
 </file>
@@ -889,476 +875,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4611B2D-2CF4-9B4C-A279-90E2C6BCED9D}">
-  <dimension ref="A1:M9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="5" max="7" width="26.6640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B1">
-        <v>1</v>
-      </c>
-      <c r="C1">
-        <v>2</v>
-      </c>
-      <c r="D1">
-        <v>3</v>
-      </c>
-      <c r="E1">
-        <v>4</v>
-      </c>
-      <c r="F1">
-        <v>5</v>
-      </c>
-      <c r="G1">
-        <v>6</v>
-      </c>
-      <c r="H1">
-        <v>7</v>
-      </c>
-      <c r="I1">
-        <v>8</v>
-      </c>
-      <c r="J1">
-        <v>9</v>
-      </c>
-      <c r="K1">
-        <v>10</v>
-      </c>
-      <c r="L1">
-        <v>11</v>
-      </c>
-      <c r="M1">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" t="s">
-        <v>62</v>
-      </c>
-      <c r="F2" t="s">
-        <v>62</v>
-      </c>
-      <c r="G2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E3" t="s">
-        <v>72</v>
-      </c>
-      <c r="F3" t="s">
-        <v>72</v>
-      </c>
-      <c r="G3" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" t="s">
-        <v>58</v>
-      </c>
-      <c r="F4" t="s">
-        <v>58</v>
-      </c>
-      <c r="G4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" t="s">
-        <v>74</v>
-      </c>
-      <c r="F5" t="s">
-        <v>74</v>
-      </c>
-      <c r="G5" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" t="s">
-        <v>63</v>
-      </c>
-      <c r="F6" t="s">
-        <v>63</v>
-      </c>
-      <c r="G6" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" t="s">
-        <v>17</v>
-      </c>
-      <c r="E7" t="s">
-        <v>73</v>
-      </c>
-      <c r="F7" t="s">
-        <v>73</v>
-      </c>
-      <c r="G7" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8" t="s">
-        <v>65</v>
-      </c>
-      <c r="F8" t="s">
-        <v>65</v>
-      </c>
-      <c r="G8" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" t="s">
-        <v>23</v>
-      </c>
-      <c r="E9" t="s">
-        <v>75</v>
-      </c>
-      <c r="F9" t="s">
-        <v>75</v>
-      </c>
-      <c r="G9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE356DF9-3DB6-A147-886E-7F10FC68241C}">
-  <dimension ref="A1:M9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="5" max="7" width="26.6640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B1">
-        <v>1</v>
-      </c>
-      <c r="C1">
-        <v>2</v>
-      </c>
-      <c r="D1">
-        <v>3</v>
-      </c>
-      <c r="E1">
-        <v>4</v>
-      </c>
-      <c r="F1">
-        <v>5</v>
-      </c>
-      <c r="G1">
-        <v>6</v>
-      </c>
-      <c r="H1">
-        <v>7</v>
-      </c>
-      <c r="I1">
-        <v>8</v>
-      </c>
-      <c r="J1">
-        <v>9</v>
-      </c>
-      <c r="K1">
-        <v>10</v>
-      </c>
-      <c r="L1">
-        <v>11</v>
-      </c>
-      <c r="M1">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" t="s">
-        <v>62</v>
-      </c>
-      <c r="F2" t="s">
-        <v>62</v>
-      </c>
-      <c r="G2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E3" t="s">
-        <v>72</v>
-      </c>
-      <c r="F3" t="s">
-        <v>72</v>
-      </c>
-      <c r="G3" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" t="s">
-        <v>58</v>
-      </c>
-      <c r="F4" t="s">
-        <v>58</v>
-      </c>
-      <c r="G4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" t="s">
-        <v>74</v>
-      </c>
-      <c r="F5" t="s">
-        <v>74</v>
-      </c>
-      <c r="G5" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" t="s">
-        <v>63</v>
-      </c>
-      <c r="F6" t="s">
-        <v>63</v>
-      </c>
-      <c r="G6" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" t="s">
-        <v>17</v>
-      </c>
-      <c r="E7" t="s">
-        <v>73</v>
-      </c>
-      <c r="F7" t="s">
-        <v>73</v>
-      </c>
-      <c r="G7" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8" t="s">
-        <v>65</v>
-      </c>
-      <c r="F8" t="s">
-        <v>65</v>
-      </c>
-      <c r="G8" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" t="s">
-        <v>23</v>
-      </c>
-      <c r="E9" t="s">
-        <v>75</v>
-      </c>
-      <c r="F9" t="s">
-        <v>75</v>
-      </c>
-      <c r="G9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A228D01-3A45-7E46-912C-9944342FCD5A}">
   <dimension ref="A1:M9"/>
@@ -3529,13 +3045,14 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A762176-A398-AB4C-A136-6BF964D77C5A}">
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="7" width="24.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="10" width="19" bestFit="1" customWidth="1"/>
+    <col min="11" max="13" width="3.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
@@ -3776,54 +3293,6 @@
       </c>
       <c r="G9" t="s">
         <v>63</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="E11" t="s">
-        <v>63</v>
-      </c>
-      <c r="F11">
-        <v>2.7320000000000002</v>
-      </c>
-      <c r="G11">
-        <f>F11/5</f>
-        <v>0.5464</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="E12" t="s">
-        <v>62</v>
-      </c>
-      <c r="F12">
-        <v>1.012</v>
-      </c>
-      <c r="G12">
-        <f t="shared" ref="G12:G14" si="0">F12/5</f>
-        <v>0.2024</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="E13" t="s">
-        <v>58</v>
-      </c>
-      <c r="F13">
-        <v>0.98899999999999999</v>
-      </c>
-      <c r="G13">
-        <f t="shared" si="0"/>
-        <v>0.1978</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="E14" t="s">
-        <v>65</v>
-      </c>
-      <c r="F14">
-        <v>1.599</v>
-      </c>
-      <c r="G14">
-        <f t="shared" si="0"/>
-        <v>0.31979999999999997</v>
       </c>
     </row>
   </sheetData>
@@ -3832,12 +3301,9 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3979,15 +3445,26 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0374E2DF-FCF3-4A80-B78B-5197E355867A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{84FF387C-D0E4-41E3-A2B6-5759715EBA83}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="399018e3-b857-408b-bd21-a6a80c979a4e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4011,17 +3488,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{84FF387C-D0E4-41E3-A2B6-5759715EBA83}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0374E2DF-FCF3-4A80-B78B-5197E355867A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="399018e3-b857-408b-bd21-a6a80c979a4e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>